<commit_message>
aligning L3stats scripts with lab style
</commit_message>
<xml_diff>
--- a/code/L3-models.xlsx
+++ b/code/L3-models.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Postdoc\Paper_brainhealth_environment\rf1-sra-environment-UG\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C252CC-2C84-4E72-9639-D12F56CEB89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F152F54-DAFF-4C1E-84FF-4F09FD9AC564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{F62FEBF3-9CDE-48EE-BCDF-3D53D9956D62}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{F62FEBF3-9CDE-48EE-BCDF-3D53D9956D62}"/>
   </bookViews>
   <sheets>
     <sheet name="adi" sheetId="1" r:id="rId1"/>
@@ -3878,8 +3878,7 @@
   <dimension ref="A1:I117"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>